<commit_message>
docs: cap nhat wireframe va dac ta Tab 2 gon gang voi 2 the KPI chinh
</commit_message>
<xml_diff>
--- a/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
+++ b/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
@@ -467,13 +467,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>I. CÁC CHỈ SỐ HÀNH VI &amp; THỜI LƯỢNG TƯƠNG TÁC NGƯỜI DÙNG (3 THẺ KPI CHÍNH TRÊN UI MỚI)</t>
+          <t>BÁO CÁO HÀNH VI &amp; THỜI LƯỢNG TƯƠNG TÁC NGƯỜI DÙNG (2 THẺ CHỈ SỐ THEO UI MỚI)</t>
         </is>
       </c>
     </row>
@@ -529,12 +529,14 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Thẻ thứ 1 (Bên trái) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
+          <t>Thẻ thứ 1 (Bên trái)
+Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>TỶ LỆ GIỮ CHÂN NGƯỜI DÙNG (Retention Rate)</t>
+          <t>TỶ LỆ GIỮ CHÂN NGƯỜI DÙNG
+(Retention Rate)</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -556,7 +558,7 @@
 Tỷ lệ giữ chân người dùng (%) = (Số lượng người dùng quay lại / Tổng số người dùng Active trong kỳ) × 100%
 • Mẫu số (Tổng người dùng Active): Số Unique Users có ít nhất 1 phiên xem phim trong kỳ lọc.
 • Tử số (Số người dùng quay lại): Số Unique Users có phát sinh xem phim ở ít nhất 2 ngày khác nhau trở lên trong kỳ lọc đã chọn.
-* Trường hợp lọc 1 ngày (D-1): Áp dụng chuẩn D1 Retention:
+* Trường hợp lọc 1 ngày (D-1): Tự động áp dụng chuẩn D1 Retention:
 Tỷ lệ D1 (%) = (Số User mới ngày D0 mở lại app ngày D+1 / Tổng User mới ngày D0) × 100%
 2. Công thức biến động so với kỳ trước:
 Biến động (%) = Tỷ lệ giữ chân kỳ này (%) - Tỷ lệ giữ chân kỳ trước liền kề (%) (Điểm phần trăm)
@@ -584,12 +586,14 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Thẻ thứ 2 (Ở giữa) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
+          <t>Thẻ thứ 2 (Bên phải)
+Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>THỜI GIAN XEM TRUNG BÌNH (Average Daily Watch Time)</t>
+          <t>THỜI GIAN XEM TRUNG BÌNH
+(Average Daily Watch Time)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -629,178 +633,8 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Thẻ thứ 3 (Bên phải) - Khối Báo Cáo Hành Vi &amp; Thời Lượng Tương Tác Người Dùng (Tab 2)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>NGƯỜI DÙNG ACTIVE (Active Users in Period)</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>124,800 Người
-▲ +12.8% so với kỳ trước
-(Phụ đề: Tổng số khán giả thực tế có xem phim trong kỳ lọc đã chọn)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Đo lường quy mô khán giả thực tế tiếp cận và tiêu thụ nội dung trên nền tảng trong khoảng thời gian được lọc.
-Đây là chỉ số nền tảng quyết định độ lớn của thị phần người xem, sức sống thực tế của ứng dụng và tiềm năng doanh thu (từ quảng cáo, lượt mở khóa tập VIP).</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>1. Công thức chỉ số chính (Người):
-Người dùng Active = COUNT(DISTINCT user_id) trong kỳ lọc đã chọn
-• Điều kiện tính: Tài khoản đăng nhập (User ID) hoặc thiết bị khách chưa đăng nhập (Device ID / UUID) có phát sinh sự kiện xem phim (Video Play) với thời lượng xem thực tế ≥ 5 giây hoặc hoàn thành ít nhất 1 tập phim.
-• Khử trùng lặp (Deduplication): Mỗi người dùng chỉ được tính 1 lần duy nhất trong toàn bộ kỳ lọc (cho dù người dùng đó xem phim ở tất cả các ngày trong kỳ).
-2. Công thức tốc độ tăng trưởng so với kỳ trước:
-Tăng trưởng (%) = [(Người dùng Active kỳ này - Người dùng Active kỳ trước) / Người dùng Active kỳ trước] × 100%
-• Ví dụ: Kỳ này 124,800 người, kỳ trước cùng độ dài đạt 110,638 người ➔ Tăng trưởng: +12.8%.</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>• Phân loại tệp người dùng:
-  - Bao gồm cả Người dùng đã đăng nhập tài khoản và Khách vãng lai (Guest xem phim qua Device ID).
-• Quy tắc hiển thị số liệu:
-  - Định dạng phân cách hàng nghìn bằng dấu phẩy kèm chữ "Người" (Ví dụ: 124,800 Người).
-• Quy tắc màu sắc biến động:
-  - Tăng trưởng dương: Hiển thị icon ▲, dấu + và màu xanh lá #00e676 (Ví dụ: ▲ +12.8% so với kỳ trước).
-  - Tăng trưởng âm: Hiển thị icon ▼, dấu - và màu đỏ #ff5252.
-  - Không đổi: 0.0% so với kỳ trước, màu xám.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>II. CÁC CHỈ SỐ PHÂN TÍCH CHUYÊN SÂU (RETENTION COHORT CHI TIẾT - PHỤC VỤ DRILL-DOWN BÁO CÁO)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Phân tích Cohort chi tiết</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>D1 Retention (Quay lại sau 1 ngày)</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>58.4%</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>Đo lường tỷ lệ người dùng mới có ấn tượng tích cực với ứng dụng và quyết định quay lại mở app xem tiếp ngay vào ngày hôm sau (D+1).</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>1. Lọc 1 ngày: Tỷ lệ D1 (%) = (Số user mới ngày D0 mở lại app vào ngày D+1 / Tổng user mới ngày D0) × 100%
-2. Lọc khoảng ngày: Là Trung bình có trọng số của các ngày trong đợt lọc đã hoàn thành chu kỳ D+1.</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>• Chuẩn ngành phim ngắn: ≥ 50% là mức Rất tốt; &lt; 40% là cảnh báo nội dung tập đầu chưa đủ cuốn hút.
-• Điều kiện: Chỉ chốt số liệu khi đã qua trọn vẹn ngày D+1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Phân tích Cohort chi tiết</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>D7 Retention (Quay lại sau 7 ngày)</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>34.8%</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>Đo lường thói quen xem phim hàng tuần của khán giả mới sau 1 tuần trải nghiệm ứng dụng (D+7).</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>1. Lọc 1 ngày: Tỷ lệ D7 (%) = (Số user mới ngày D0 còn quay lại vào ngày D+7 / Tổng user mới ngày D0) × 100%
-2. Lọc khoảng ngày: Là Trung bình có trọng số của các nhóm user đã trải qua đủ 7 ngày tuổi tính đến hiện tại.</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>• Chuẩn ngành: Đạt từ 30% đến 40% là Tốt.
-• Ngày chưa đủ hạn 7 ngày sẽ không đưa vào mẫu số để tránh làm sai lệch tỷ lệ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Phân tích Cohort chi tiết</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>D30 Retention (Quay lại sau 30 ngày)</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>21.2%</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Tỷ lệ khán giả trung thành cốt lõi còn gắn bó với ứng dụng sau 1 tháng sử dụng (D+30), mang lại giá trị vòng đời (LTV) lâu dài.</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>1. Lọc 1 ngày: Tỷ lệ D30 (%) = (Số user mới ngày D0 mở lại app ngày D+30 / Tổng user mới ngày D0) × 100%
-2. Lọc khoảng ngày: Trung bình có trọng số của các nhóm user đã trải qua đủ 30 ngày tuổi tính đến hiện tại.</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>• Chuẩn ngành: ≥ 20% là mức xuất sắc cho ứng dụng phim ngắn.
-• Nếu chưa đủ 30 ngày so với hiện tại: Hiển thị dấu gạch ngang "--" (Đang tích lũy chu kỳ), tuyệt đối không để 0% hoặc NaN.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A6:G6"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: bo sung vi du tinh toan chi tiet cho Ty le giu chan va Thoi gian xem TB
</commit_message>
<xml_diff>
--- a/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
+++ b/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
@@ -475,7 +475,7 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -554,15 +554,30 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>1. Công thức chỉ số chính (%):
+          <t>1. CÔNG THỨC CHỈ SỐ CHÍNH (%):
 Tỷ lệ giữ chân người dùng (%) = (Số lượng người dùng quay lại / Tổng số người dùng Active trong kỳ) × 100%
 • Mẫu số (Tổng người dùng Active): Số Unique Users có ít nhất 1 phiên xem phim trong kỳ lọc.
 • Tử số (Số người dùng quay lại): Số Unique Users có phát sinh xem phim ở ít nhất 2 ngày khác nhau trở lên trong kỳ lọc đã chọn.
-* Trường hợp lọc 1 ngày (D-1): Tự động áp dụng chuẩn D1 Retention:
+────────────────────────────────────────
+► VÍ DỤ 1: KHI LỌC KHOẢNG NGÀY (VD: Kỳ lọc 11 ngày từ 10/08 đến 20/08):
+- Mẫu số: Toàn bộ 11 ngày có 100,000 khán giả duy nhất (Unique Users) có mở xem phim.
+- Tử số: Trong 100,000 khán giả đó, có 58,400 người có xem phim ở từ 2 ngày khác nhau trở lên trong kỳ (VD: xem ngày 10/08 và quay lại xem tiếp ngày 12/08...).
+➔ Tỷ lệ giữ chân = (58,400 / 100,000) × 100% = 58.4%.
+(41,600 người còn lại chỉ vào xem 1 ngày duy nhất rồi chưa quay lại).
+────────────────────────────────────────
+► VÍ DỤ 2: KHI LỌC 1 NGÀY (D-1 mặc định, VD: Ngày 10/08):
+Tự động áp dụng chuẩn D1 Retention Cohort (Giữ chân sau 24h):
 Tỷ lệ D1 (%) = (Số User mới ngày D0 mở lại app ngày D+1 / Tổng User mới ngày D0) × 100%
-2. Công thức biến động so với kỳ trước:
-Biến động (%) = Tỷ lệ giữ chân kỳ này (%) - Tỷ lệ giữ chân kỳ trước liền kề (%) (Điểm phần trăm)
-• Ví dụ: Kỳ này (10/08 - 20/08: 11 ngày) đạt 58.4%, kỳ liền kề trước đó (30/07 - 09/08: 11 ngày) đạt 54.2% ➔ Biến động: +4.2%</t>
+- Mẫu số: Ngày 10/08 (D0) có 10,000 người dùng mới cài app &amp; xem phim lần đầu.
+- Tử số: Sang ngày 11/08 (D+1), có 5,840 người trong nhóm đó quay lại mở app xem tiếp.
+➔ Tỷ lệ D1 = (5,840 / 10,000) × 100% = 58.4%.
+────────────────────────────────────────
+2. CÔNG THỨC BIẾN ĐỘNG SO VỚI KỲ TRƯỚC:
+Biến động (%) = Tỷ lệ giữ chân kỳ này (%) - Tỷ lệ giữ chân kỳ trước liền kề (%)
+► VÍ DỤ 3: TÍNH BIẾN ĐỘNG:
+- Kỳ này (10/08 - 20/08: 11 ngày): Đạt 58.4%.
+- Kỳ trước liền kề (30/07 - 09/08: cùng 11 ngày): Đạt 54.2%.
+➔ Biến động = 58.4% - 54.2% = +4.2% (Hiển thị icon ▲ +4.2% so với kỳ trước).</t>
         </is>
       </c>
       <c r="G3" s="4" t="inlineStr">
@@ -611,14 +626,21 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>1. Công thức chỉ số chính (Phút/Ngày):
+          <t>1. CÔNG THỨC CHỈ SỐ CHÍNH (Phút/Ngày):
 Thời gian xem TB (Phút/Ngày) = (Tổng số phút xem video của tất cả người dùng trong kỳ) / (Tổng số lượt User-Day hoạt động trong kỳ)
 • Tổng số phút xem: Tổng thời lượng phát video thực tế của tất cả khán giả trong kỳ (quy đổi ra phút).
 • Tổng số lượt User-Day: Tổng cộng số ngày có xem phim của từng người dùng trong kỳ (Mỗi User xem trong 1 ngày = 1 User-Day).
-• Ví dụ: Trong kỳ lọc 11 ngày, hệ thống ghi nhận tổng 6,052,800 phút xem phim qua 124,800 lượt User-Day ➔ Thời gian xem TB = 6,052,800 / 124,800 = 48.5 Phút/Ngày.
-2. Công thức biến động so với kỳ trước:
+────────────────────────────────────────
+► VÍ DỤ MINH HỌA:
+- Trong kỳ lọc 11 ngày (10/08 - 20/08), hệ thống ghi nhận:
+  + Tổng số phút xem phim tích lũy toàn hệ thống = 6,052,800 phút.
+  + Tổng số lượt khán giả hoạt động (User-Day) = 124,800 lượt.
+➔ Thời gian xem TB = 6,052,800 / 124,800 = 48.5 Phút / Ngày.
+────────────────────────────────────────
+2. CÔNG THỨC BIẾN ĐỘNG SO VỚI KỲ TRƯỚC:
 Biến động (phút) = Thời gian xem TB kỳ này - Thời gian xem TB kỳ trước liền kề
-• Ví dụ: Kỳ này 48.5 phút/ngày, kỳ trước 42.0 phút/ngày ➔ Biến động: +6.5 phút.</t>
+- Kỳ này đạt 48.5 phút/ngày; kỳ trước liền kề đạt 42.0 phút/ngày.
+➔ Biến động = 48.5 - 42.0 = +6.5 phút (Hiển thị icon ▲ +6.5 phút so với kỳ trước).</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">

</xml_diff>

<commit_message>
docs: chuan hoa logic D1 khi loc 1 ngay theo goc nhin van hanh thuc te
</commit_message>
<xml_diff>
--- a/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
+++ b/result_docs/Bang_Dac_Ta_Tab2_Bao_Cao_Hanh_Vi_User.xlsx
@@ -475,7 +475,7 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="65" customWidth="1" min="6" max="6"/>
     <col width="48" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -556,25 +556,27 @@
         <is>
           <t>1. CÔNG THỨC CHỈ SỐ CHÍNH (%):
 Tỷ lệ giữ chân người dùng (%) = (Số lượng người dùng quay lại / Tổng số người dùng Active trong kỳ) × 100%
-• Mẫu số (Tổng người dùng Active): Số Unique Users có ít nhất 1 phiên xem phim trong kỳ lọc.
-• Tử số (Số người dùng quay lại): Số Unique Users có phát sinh xem phim ở ít nhất 2 ngày khác nhau trở lên trong kỳ lọc đã chọn.
 ────────────────────────────────────────
-► VÍ DỤ 1: KHI LỌC KHOẢNG NGÀY (VD: Kỳ lọc 11 ngày từ 10/08 đến 20/08):
-- Mẫu số: Toàn bộ 11 ngày có 100,000 khán giả duy nhất (Unique Users) có mở xem phim.
-- Tử số: Trong 100,000 khán giả đó, có 58,400 người có xem phim ở từ 2 ngày khác nhau trở lên trong kỳ (VD: xem ngày 10/08 và quay lại xem tiếp ngày 12/08...).
-➔ Tỷ lệ giữ chân = (58,400 / 100,000) × 100% = 58.4%.
-(41,600 người còn lại chỉ vào xem 1 ngày duy nhất rồi chưa quay lại).
+► TRƯỜNG HỢP 1: KHI LỌC 1 NGÀY (VD: Lọc ngày 10/08)
+Áp dụng chuẩn D1 Retention (Đo lường năng lực kéo người dùng hôm qua quay lại hôm nay):
+• Mẫu số: Tổng số người dùng mới cài app &amp; xem phim vào ngày hôm trước (Ngày 09/08).
+• Tử số: Số người dùng mới của ngày 09/08 có quay lại mở app xem tiếp vào chính ngày đang lọc (Ngày 10/08).
+Ví dụ minh họa:
+- Ngày hôm trước (09/08): Hệ thống đón 10,000 người dùng mới (Mẫu số = 10,000).
+- Ngày đang lọc (10/08): Trong 10,000 người đó, có 5,840 người quay lại mở app xem tiếp (Tử số = 5,840).
+➔ Tỷ lệ D1 ngày 10/08 = (5,840 / 10,000) × 100% = 58.4%.
+* Ưu điểm nghiệp vụ: Số liệu chốt ngay trong ngày 10/08, người xem filter ngày 10/08 là có ngay số liệu thực tế mà không cần đợi sang ngày 11/08!
 ────────────────────────────────────────
-► VÍ DỤ 2: KHI LỌC 1 NGÀY (D-1 mặc định, VD: Ngày 10/08):
-Tự động áp dụng chuẩn D1 Retention Cohort (Giữ chân sau 24h):
-Tỷ lệ D1 (%) = (Số User mới ngày D0 mở lại app ngày D+1 / Tổng User mới ngày D0) × 100%
-- Mẫu số: Ngày 10/08 (D0) có 10,000 người dùng mới cài app &amp; xem phim lần đầu.
-- Tử số: Sang ngày 11/08 (D+1), có 5,840 người trong nhóm đó quay lại mở app xem tiếp.
-➔ Tỷ lệ D1 = (5,840 / 10,000) × 100% = 58.4%.
+► TRƯỜNG HỢP 2: KHI LỌC KHOẢNG NGÀY (VD: Kỳ lọc 11 ngày từ 10/08 đến 20/08)
+Tỷ lệ giữ chân trong kỳ (%) = (Số Unique Users quay lại / Tổng Unique Users Active trong kỳ) × 100%
+- Mẫu số (Tổng Active trong kỳ): Toàn bộ 11 ngày có 100,000 khán giả duy nhất (Unique Users) có mở xem phim.
+- Tử số (Số người quay lại): Trong 100,000 khán giả đó, có 58,400 người có xem phim ở từ 2 ngày khác nhau trở lên trong kỳ (VD: xem ngày 10/08 và xem tiếp ngày 12/08...).
+➔ Tỷ lệ giữ chân cả kỳ = (58,400 / 100,000) × 100% = 58.4%.
+(41,600 người còn lại chỉ vào xem 1 ngày duy nhất trong cả kỳ lọc rồi chưa quay lại).
 ────────────────────────────────────────
 2. CÔNG THỨC BIẾN ĐỘNG SO VỚI KỲ TRƯỚC:
 Biến động (%) = Tỷ lệ giữ chân kỳ này (%) - Tỷ lệ giữ chân kỳ trước liền kề (%)
-► VÍ DỤ 3: TÍNH BIẾN ĐỘNG:
+► Ví dụ:
 - Kỳ này (10/08 - 20/08: 11 ngày): Đạt 58.4%.
 - Kỳ trước liền kề (30/07 - 09/08: cùng 11 ngày): Đạt 54.2%.
 ➔ Biến động = 58.4% - 54.2% = +4.2% (Hiển thị icon ▲ +4.2% so với kỳ trước).</t>
@@ -590,7 +592,9 @@
   - Tăng: Icon ▲ kèm dấu + và giá trị, màu xanh lá.
   - Giảm: Icon ▼ kèm dấu - và giá trị, màu đỏ.
   - Bằng nhau: 0.0% so với kỳ trước, màu xám.
-• Điều kiện chốt số liệu: Dữ liệu giữ chân người dùng chỉ chốt số trọn vẹn sau khi kết thúc 23:59:59 của ngày cuối cùng trong kỳ lọc.
+• Điều kiện chốt số liệu:
+  - Khi lọc 1 ngày (10/08): Số liệu D1 được chốt hoàn tất vào cuối ngày 10/08 (23:59:59).
+  - Khi lọc khoảng ngày: Dữ liệu chốt sau khi kết thúc ngày cuối cùng của kỳ lọc.
 • Làm tròn: Làm tròn 1 chữ số thập phân (Ví dụ: 58.4%).</t>
         </is>
       </c>

</xml_diff>